<commit_message>
Evidencias: ajustes de la rama claude/guias-digemid (periodo, lote/vencimiento, sugeridas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TRpE1oShihdbrH9mzx317w
</commit_message>
<xml_diff>
--- a/capturas_guias_digemid/dig_digemid.xlsx
+++ b/capturas_guias_digemid/dig_digemid.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:X11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -405,22 +405,24 @@
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
     <col min="9" max="9" width="30.83203125" customWidth="1"/>
     <col min="10" max="10" width="30.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="30.83203125" customWidth="1"/>
     <col min="12" max="12" width="36.83203125" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" customWidth="1"/>
-    <col min="14" max="14" width="40.83203125" customWidth="1"/>
-    <col min="15" max="15" width="8.83203125" customWidth="1"/>
-    <col min="16" max="16" width="9.83203125" customWidth="1"/>
-    <col min="17" max="17" width="6.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="36.83203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="15" max="15" width="40.83203125" customWidth="1"/>
+    <col min="16" max="16" width="8.83203125" customWidth="1"/>
+    <col min="17" max="17" width="9.83203125" customWidth="1"/>
+    <col min="18" max="18" width="6.83203125" customWidth="1"/>
     <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
-    <col min="21" max="21" width="16.83203125" customWidth="1"/>
-    <col min="22" max="22" width="40.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" customWidth="1"/>
+    <col min="22" max="22" width="16.83203125" customWidth="1"/>
+    <col min="23" max="23" width="16.83203125" customWidth="1"/>
+    <col min="24" max="24" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -443,51 +445,57 @@
         <v>Factura vinculada</v>
       </c>
       <c r="G1" t="str">
+        <v>Factura sugerida (según nota, sin vincular)</v>
+      </c>
+      <c r="H1" t="str">
         <v>RUC</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Cliente</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Almacén de salida</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Almacén de destino</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Punto de partida</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Punto de llegada</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Código</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Producto</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Producto DIGEMID</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Cantidad</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Unidad</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Lote</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
+        <v>Fecha de fabricación</v>
+      </c>
+      <c r="U1" t="str">
         <v>Fecha de vencimiento</v>
       </c>
-      <c r="T1" t="str">
+      <c r="V1" t="str">
         <v>Registro sanitario</v>
       </c>
-      <c r="U1" t="str">
+      <c r="W1" t="str">
         <v>Estado de la guía</v>
       </c>
-      <c r="V1" t="str">
+      <c r="X1" t="str">
         <v>Enlace PDF</v>
       </c>
     </row>
@@ -511,51 +519,57 @@
         <v>F001-000001</v>
       </c>
       <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v>20111111111</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>CLINICA UNO SAC</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>ALMACEN PRINCIPAL - Av. Almacen 500, Ate</v>
       </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v>Partida de TTT1-000001 (150103)</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>Llegada de TTT1-000001 (150131)</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>D001</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>GUANTE NITRILO M R.S. DM-12345-E LOTE A123 F.V. 12/2027</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>Sí</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>5</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="R2" t="str">
         <v>NIU</v>
       </c>
-      <c r="R2" t="str">
+      <c r="S2" t="str">
         <v>A123</v>
       </c>
-      <c r="S2" t="str">
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
         <v>12/2027</v>
       </c>
-      <c r="T2" t="str">
+      <c r="V2" t="str">
         <v>DM-12345-E</v>
       </c>
-      <c r="U2" t="str">
+      <c r="W2" t="str">
         <v>Facturada</v>
       </c>
-      <c r="V2" t="str">
+      <c r="X2" t="str">
         <v>https://nube.test/pdf/TTT1-000001.pdf</v>
       </c>
     </row>
@@ -579,51 +593,57 @@
         <v/>
       </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
         <v>20222222222</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>BOTICA DOS EIRL</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>ALMACEN PRINCIPAL - Av. Almacen 500, Ate</v>
       </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
       <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
         <v>Partida de TTT1-000004 (150103)</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Llegada de TTT1-000004 (150131)</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>D002</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v>MASCARILLA KN95</v>
       </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
         <v>Sí</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>1</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="R3" t="str">
         <v>NIU</v>
       </c>
-      <c r="R3" t="str">
-        <v/>
-      </c>
       <c r="S3" t="str">
         <v/>
       </c>
       <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
         <v>DM7788E</v>
       </c>
-      <c r="U3" t="str">
+      <c r="W3" t="str">
         <v>De baja (interna)</v>
       </c>
-      <c r="V3" t="str">
+      <c r="X3" t="str">
         <v>https://nube.test/pdf/TTT1-000004.pdf</v>
       </c>
     </row>
@@ -647,51 +667,57 @@
         <v>F001-000002</v>
       </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
         <v>20111111111</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>CLINICA UNO SAC</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
       <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
         <v>Partida de TTT4-000001 (150103)</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>Llegada de TTT4-000001 (150131)</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>D001</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>GUANTE NITRILO M R.S. DM-12345-E LOTE A123 F.V. 12/2027</v>
       </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
         <v>Sí</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>2</v>
       </c>
-      <c r="Q4" t="str">
+      <c r="R4" t="str">
         <v>NIU</v>
       </c>
-      <c r="R4" t="str">
+      <c r="S4" t="str">
         <v>A123</v>
       </c>
-      <c r="S4" t="str">
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
         <v>12/2027</v>
       </c>
-      <c r="T4" t="str">
+      <c r="V4" t="str">
         <v>DM-12345-E</v>
       </c>
-      <c r="U4" t="str">
+      <c r="W4" t="str">
         <v>Facturada</v>
       </c>
-      <c r="V4" t="str">
+      <c r="X4" t="str">
         <v>https://nube.test/pdf/TTT4-000001.pdf</v>
       </c>
     </row>
@@ -715,51 +741,57 @@
         <v/>
       </c>
       <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
         <v>20222222222</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>BOTICA DOS EIRL</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
       </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
       <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
         <v>Partida de TTT4-000003 (150103)</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
         <v>Llegada de TTT4-000003 (150131)</v>
       </c>
-      <c r="M5" t="str">
+      <c r="N5" t="str">
         <v>D002</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v>MASCARILLA KN95</v>
       </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
         <v>Sí</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>1</v>
       </c>
-      <c r="Q5" t="str">
+      <c r="R5" t="str">
         <v>NIU</v>
       </c>
-      <c r="R5" t="str">
-        <v/>
-      </c>
       <c r="S5" t="str">
         <v/>
       </c>
       <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
         <v>DM7788E</v>
       </c>
-      <c r="U5" t="str">
+      <c r="W5" t="str">
         <v>Anulada (SUNAT)</v>
       </c>
-      <c r="V5" t="str">
+      <c r="X5" t="str">
         <v>https://nube.test/pdf/TTT4-000003.pdf</v>
       </c>
     </row>
@@ -783,64 +815,445 @@
         <v/>
       </c>
       <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
         <v>20222222222</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>BOTICA DOS EIRL</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
       <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
         <v>Partida de TTT4-000002 (150103)</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
         <v>Llegada de TTT4-000002 (150131)</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>D002</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>MASCARILLA KN95</v>
       </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
         <v>Sí</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>4</v>
       </c>
-      <c r="Q6" t="str">
+      <c r="R6" t="str">
         <v>NIU</v>
       </c>
-      <c r="R6" t="str">
-        <v/>
-      </c>
       <c r="S6" t="str">
         <v/>
       </c>
       <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
         <v>DM7788E</v>
       </c>
-      <c r="U6" t="str">
+      <c r="W6" t="str">
         <v>Emitida</v>
       </c>
-      <c r="V6" t="str">
+      <c r="X6" t="str">
         <v>https://nube.test/pdf/TTT4-000002.pdf</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>TTT4</v>
+      </c>
+      <c r="C7" t="str">
+        <v>000010</v>
+      </c>
+      <c r="D7" t="str">
+        <v>TTT4-000010</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Parte DIGEMID</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>F001-000007</v>
+      </c>
+      <c r="H7" t="str">
+        <v>20222222222</v>
+      </c>
+      <c r="I7" t="str">
+        <v>BOTICA DOS EIRL</v>
+      </c>
+      <c r="J7" t="str">
+        <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v>Partida de TTT4-000010 (150103)</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Llegada de TTT4-000010 (150131)</v>
+      </c>
+      <c r="N7" t="str">
+        <v>D006</v>
+      </c>
+      <c r="O7" t="str">
+        <v>ALCOHOL ETILICO 70 GRADOS 1 LT</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="Q7">
+        <v>2</v>
+      </c>
+      <c r="R7" t="str">
+        <v>NIU</v>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v>Emitida</v>
+      </c>
+      <c r="X7" t="str">
+        <v>https://nube.test/pdf/TTT4-000010.pdf</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>TTT4</v>
+      </c>
+      <c r="C8" t="str">
+        <v>000010</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TTT4-000010</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Parte DIGEMID</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>F001-000007</v>
+      </c>
+      <c r="H8" t="str">
+        <v>20222222222</v>
+      </c>
+      <c r="I8" t="str">
+        <v>BOTICA DOS EIRL</v>
+      </c>
+      <c r="J8" t="str">
+        <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v>Partida de TTT4-000010 (150103)</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Llegada de TTT4-000010 (150131)</v>
+      </c>
+      <c r="N8" t="str">
+        <v>D003</v>
+      </c>
+      <c r="O8" t="str">
+        <v>GUANTE DE NITRILO AZUL X 100 UNID 3.5 GRAMOS F.F 01-2026 F.V</v>
+      </c>
+      <c r="P8" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="Q8">
+        <v>2</v>
+      </c>
+      <c r="R8" t="str">
+        <v>NIU</v>
+      </c>
+      <c r="S8" t="str">
+        <v>IN25029097</v>
+      </c>
+      <c r="T8" t="str">
+        <v>01-2026</v>
+      </c>
+      <c r="U8" t="str">
+        <v>01-2029</v>
+      </c>
+      <c r="V8" t="str">
+        <v>DM-10293-E</v>
+      </c>
+      <c r="W8" t="str">
+        <v>Emitida</v>
+      </c>
+      <c r="X8" t="str">
+        <v>https://nube.test/pdf/TTT4-000010.pdf</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>TTT4</v>
+      </c>
+      <c r="C9" t="str">
+        <v>000010</v>
+      </c>
+      <c r="D9" t="str">
+        <v>TTT4-000010</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Parte DIGEMID</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>F001-000007</v>
+      </c>
+      <c r="H9" t="str">
+        <v>20222222222</v>
+      </c>
+      <c r="I9" t="str">
+        <v>BOTICA DOS EIRL</v>
+      </c>
+      <c r="J9" t="str">
+        <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v>Partida de TTT4-000010 (150103)</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Llegada de TTT4-000010 (150131)</v>
+      </c>
+      <c r="N9" t="str">
+        <v>D005</v>
+      </c>
+      <c r="O9" t="str">
+        <v xml:space="preserve">JERINGA DESCARTABLE 5ML C/AGUJA 21G X 100 UNID LTE. 2405117 </v>
+      </c>
+      <c r="P9" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="Q9">
+        <v>2</v>
+      </c>
+      <c r="R9" t="str">
+        <v>NIU</v>
+      </c>
+      <c r="S9" t="str">
+        <v>2405117</v>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v>05/2029</v>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v>Emitida</v>
+      </c>
+      <c r="X9" t="str">
+        <v>https://nube.test/pdf/TTT4-000010.pdf</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>TTT4</v>
+      </c>
+      <c r="C10" t="str">
+        <v>000010</v>
+      </c>
+      <c r="D10" t="str">
+        <v>TTT4-000010</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Parte DIGEMID</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v>F001-000007</v>
+      </c>
+      <c r="H10" t="str">
+        <v>20222222222</v>
+      </c>
+      <c r="I10" t="str">
+        <v>BOTICA DOS EIRL</v>
+      </c>
+      <c r="J10" t="str">
+        <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v>Partida de TTT4-000010 (150103)</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Llegada de TTT4-000010 (150131)</v>
+      </c>
+      <c r="N10" t="str">
+        <v>D004</v>
+      </c>
+      <c r="O10" t="str">
+        <v xml:space="preserve">MASCARILLA QUIRURGICA 3 PLIEGUES X 50 UNID LTE. MQ2408 F.F. </v>
+      </c>
+      <c r="P10" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="Q10">
+        <v>2</v>
+      </c>
+      <c r="R10" t="str">
+        <v>NIU</v>
+      </c>
+      <c r="S10" t="str">
+        <v>MQ2408</v>
+      </c>
+      <c r="T10" t="str">
+        <v>08-2024</v>
+      </c>
+      <c r="U10" t="str">
+        <v>08-2027</v>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v>Emitida</v>
+      </c>
+      <c r="X10" t="str">
+        <v>https://nube.test/pdf/TTT4-000010.pdf</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>TTT4</v>
+      </c>
+      <c r="C11" t="str">
+        <v>000010</v>
+      </c>
+      <c r="D11" t="str">
+        <v>TTT4-000010</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Parte DIGEMID</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v>F001-000007</v>
+      </c>
+      <c r="H11" t="str">
+        <v>20222222222</v>
+      </c>
+      <c r="I11" t="str">
+        <v>BOTICA DOS EIRL</v>
+      </c>
+      <c r="J11" t="str">
+        <v>ALMACEN DIGEMID - Calle Sanitaria 20, Lima</v>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v>Partida de TTT4-000010 (150103)</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Llegada de TTT4-000010 (150131)</v>
+      </c>
+      <c r="N11" t="str">
+        <v>D007</v>
+      </c>
+      <c r="O11" t="str">
+        <v xml:space="preserve">GASA ESTERIL 10X10 CM X 100 SOBRES LOTE SIN NUMERO F.V. VER </v>
+      </c>
+      <c r="P11" t="str">
+        <v>Sí</v>
+      </c>
+      <c r="Q11">
+        <v>2</v>
+      </c>
+      <c r="R11" t="str">
+        <v>NIU</v>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v>Emitida</v>
+      </c>
+      <c r="X11" t="str">
+        <v>https://nube.test/pdf/TTT4-000010.pdf</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="V2" r:id="rId1"/>
-    <hyperlink ref="V3" r:id="rId2"/>
-    <hyperlink ref="V4" r:id="rId3"/>
-    <hyperlink ref="V5" r:id="rId4"/>
-    <hyperlink ref="V6" r:id="rId5"/>
+    <hyperlink ref="X2" r:id="rId1"/>
+    <hyperlink ref="X3" r:id="rId2"/>
+    <hyperlink ref="X4" r:id="rId3"/>
+    <hyperlink ref="X5" r:id="rId4"/>
+    <hyperlink ref="X6" r:id="rId5"/>
+    <hyperlink ref="X7" r:id="rId6"/>
+    <hyperlink ref="X8" r:id="rId7"/>
+    <hyperlink ref="X9" r:id="rId8"/>
+    <hyperlink ref="X10" r:id="rId9"/>
+    <hyperlink ref="X11" r:id="rId10"/>
   </hyperlinks>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>